<commit_message>
Prepare SharePoint workbook integration
</commit_message>
<xml_diff>
--- a/deliverables/Prime_Control_Respostas_NPS_2026_Modelo_SharePoint.xlsx
+++ b/deliverables/Prime_Control_Respostas_NPS_2026_Modelo_SharePoint.xlsx
@@ -40,6 +40,11 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <color rgb="00172B4D"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="000E243D"/>
       <sz val="24"/>
@@ -66,11 +71,6 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <color rgb="00172B4D"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -135,21 +135,21 @@
   </cellStyleXfs>
   <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="9" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -158,13 +158,13 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -406,6 +406,60 @@
     <clientData/>
   </oneCellAnchor>
 </wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRespostasNPS" displayName="TabelaRespostasNPS" ref="A1:AS2" headerRowCount="1">
+  <autoFilter ref="A1:AS2"/>
+  <tableColumns count="45">
+    <tableColumn id="1" name="ID resposta"/>
+    <tableColumn id="2" name="Data de resposta"/>
+    <tableColumn id="3" name="Campanha"/>
+    <tableColumn id="4" name="Status"/>
+    <tableColumn id="5" name="Fonte"/>
+    <tableColumn id="6" name="Token / sessão"/>
+    <tableColumn id="7" name="Empresa"/>
+    <tableColumn id="8" name="Nome"/>
+    <tableColumn id="9" name="E-mail corporativo"/>
+    <tableColumn id="10" name="Cargo"/>
+    <tableColumn id="11" name="Responsável Prime Control"/>
+    <tableColumn id="12" name="Início"/>
+    <tableColumn id="13" name="Conclusão"/>
+    <tableColumn id="14" name="Tempo de conclusão (min)"/>
+    <tableColumn id="15" name="Dispositivo"/>
+    <tableColumn id="16" name="Navegador"/>
+    <tableColumn id="17" name="Nota NPS (1 a 10)"/>
+    <tableColumn id="18" name="Classificação NPS"/>
+    <tableColumn id="19" name="Motivo da nota"/>
+    <tableColumn id="20" name="Entendimento do negócio"/>
+    <tableColumn id="21" name="Relevância das soluções entregues"/>
+    <tableColumn id="22" name="Valor percebido"/>
+    <tableColumn id="23" name="Comprometimento com resultados"/>
+    <tableColumn id="24" name="Engajamento na solução de problemas"/>
+    <tableColumn id="25" name="Qualidade das entregas"/>
+    <tableColumn id="26" name="Cumprimento dos prazos"/>
+    <tableColumn id="27" name="Clareza e objetividade"/>
+    <tableColumn id="28" name="Tempo de resposta da equipe"/>
+    <tableColumn id="29" name="Qualidade do atendimento"/>
+    <tableColumn id="30" name="Empresa inovadora e alinhada ao mercado"/>
+    <tableColumn id="31" name="Antecipar tendências e propor soluções"/>
+    <tableColumn id="32" name="Áreas para investir mais em inovação"/>
+    <tableColumn id="33" name="Expectativa sobre parceria estratégica"/>
+    <tableColumn id="34" name="Iniciativas/melhorias para gerar mais valor"/>
+    <tableColumn id="35" name="Perguntas respondidas"/>
+    <tableColumn id="36" name="Campos abertos preenchidos"/>
+    <tableColumn id="37" name="Etapa abandonada"/>
+    <tableColumn id="38" name="Sinal de risco"/>
+    <tableColumn id="39" name="Status de follow-up"/>
+    <tableColumn id="40" name="Próxima ação"/>
+    <tableColumn id="41" name="Responsável follow-up"/>
+    <tableColumn id="42" name="Data follow-up"/>
+    <tableColumn id="43" name="Observações internas"/>
+    <tableColumn id="44" name="Link replay Clarity (opcional)"/>
+    <tableColumn id="45" name="Última atualização"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1063,7 +1117,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS1"/>
+  <dimension ref="A1:AS2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1340,6 +1394,53 @@
         </is>
       </c>
     </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="10" t="inlineStr"/>
+      <c r="B2" s="10" t="inlineStr"/>
+      <c r="C2" s="10" t="inlineStr"/>
+      <c r="D2" s="10" t="inlineStr"/>
+      <c r="E2" s="10" t="inlineStr"/>
+      <c r="F2" s="10" t="inlineStr"/>
+      <c r="G2" s="10" t="inlineStr"/>
+      <c r="H2" s="10" t="inlineStr"/>
+      <c r="I2" s="10" t="inlineStr"/>
+      <c r="J2" s="10" t="inlineStr"/>
+      <c r="K2" s="10" t="inlineStr"/>
+      <c r="L2" s="10" t="inlineStr"/>
+      <c r="M2" s="10" t="inlineStr"/>
+      <c r="N2" s="10" t="inlineStr"/>
+      <c r="O2" s="10" t="inlineStr"/>
+      <c r="P2" s="10" t="inlineStr"/>
+      <c r="Q2" s="10" t="inlineStr"/>
+      <c r="R2" s="10" t="inlineStr"/>
+      <c r="S2" s="10" t="inlineStr"/>
+      <c r="T2" s="10" t="inlineStr"/>
+      <c r="U2" s="10" t="inlineStr"/>
+      <c r="V2" s="10" t="inlineStr"/>
+      <c r="W2" s="10" t="inlineStr"/>
+      <c r="X2" s="10" t="inlineStr"/>
+      <c r="Y2" s="10" t="inlineStr"/>
+      <c r="Z2" s="10" t="inlineStr"/>
+      <c r="AA2" s="10" t="inlineStr"/>
+      <c r="AB2" s="10" t="inlineStr"/>
+      <c r="AC2" s="10" t="inlineStr"/>
+      <c r="AD2" s="10" t="inlineStr"/>
+      <c r="AE2" s="10" t="inlineStr"/>
+      <c r="AF2" s="10" t="inlineStr"/>
+      <c r="AG2" s="10" t="inlineStr"/>
+      <c r="AH2" s="10" t="inlineStr"/>
+      <c r="AI2" s="10" t="inlineStr"/>
+      <c r="AJ2" s="10" t="inlineStr"/>
+      <c r="AK2" s="10" t="inlineStr"/>
+      <c r="AL2" s="10" t="inlineStr"/>
+      <c r="AM2" s="10" t="inlineStr"/>
+      <c r="AN2" s="10" t="inlineStr"/>
+      <c r="AO2" s="10" t="inlineStr"/>
+      <c r="AP2" s="10" t="inlineStr"/>
+      <c r="AQ2" s="10" t="inlineStr"/>
+      <c r="AR2" s="10" t="inlineStr"/>
+      <c r="AS2" s="10" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:AS1"/>
   <conditionalFormatting sqref="Q2:Q5000">
@@ -1372,6 +1473,9 @@
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Update 2026 survey questions and archive 2027 version
</commit_message>
<xml_diff>
--- a/deliverables/Prime_Control_Respostas_NPS_2026_Modelo_SharePoint.xlsx
+++ b/deliverables/Prime_Control_Respostas_NPS_2026_Modelo_SharePoint.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dicionário" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base automática'!$A$1:$AS$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Base automática'!$A$1:$AQ$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -409,9 +409,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRespostasNPS" displayName="TabelaRespostasNPS" ref="A1:AS2" headerRowCount="1">
-  <autoFilter ref="A1:AS2"/>
-  <tableColumns count="45">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="TabelaRespostasNPS" displayName="TabelaRespostasNPS" ref="A1:AQ2" headerRowCount="1">
+  <autoFilter ref="A1:AQ2"/>
+  <tableColumns count="43">
     <tableColumn id="1" name="ID resposta"/>
     <tableColumn id="2" name="Data de resposta"/>
     <tableColumn id="3" name="Campanha"/>
@@ -428,35 +428,33 @@
     <tableColumn id="14" name="Tempo de conclusão (min)"/>
     <tableColumn id="15" name="Dispositivo"/>
     <tableColumn id="16" name="Navegador"/>
-    <tableColumn id="17" name="Nota NPS (1 a 10)"/>
+    <tableColumn id="17" name="Nota NPS (0 a 10)"/>
     <tableColumn id="18" name="Classificação NPS"/>
-    <tableColumn id="19" name="Motivo da nota"/>
-    <tableColumn id="20" name="Entendimento do negócio"/>
-    <tableColumn id="21" name="Relevância das soluções entregues"/>
-    <tableColumn id="22" name="Valor percebido"/>
-    <tableColumn id="23" name="Comprometimento com resultados"/>
-    <tableColumn id="24" name="Engajamento na solução de problemas"/>
-    <tableColumn id="25" name="Qualidade das entregas"/>
-    <tableColumn id="26" name="Cumprimento dos prazos"/>
-    <tableColumn id="27" name="Clareza e objetividade"/>
-    <tableColumn id="28" name="Tempo de resposta da equipe"/>
-    <tableColumn id="29" name="Qualidade do atendimento"/>
-    <tableColumn id="30" name="Empresa inovadora e alinhada ao mercado"/>
-    <tableColumn id="31" name="Antecipar tendências e propor soluções"/>
-    <tableColumn id="32" name="Áreas para investir mais em inovação"/>
-    <tableColumn id="33" name="Expectativa sobre parceria estratégica"/>
-    <tableColumn id="34" name="Iniciativas/melhorias para gerar mais valor"/>
-    <tableColumn id="35" name="Perguntas respondidas"/>
-    <tableColumn id="36" name="Campos abertos preenchidos"/>
-    <tableColumn id="37" name="Etapa abandonada"/>
-    <tableColumn id="38" name="Sinal de risco"/>
-    <tableColumn id="39" name="Status de follow-up"/>
-    <tableColumn id="40" name="Próxima ação"/>
-    <tableColumn id="41" name="Responsável follow-up"/>
-    <tableColumn id="42" name="Data follow-up"/>
-    <tableColumn id="43" name="Observações internas"/>
-    <tableColumn id="44" name="Link replay Clarity (opcional)"/>
-    <tableColumn id="45" name="Última atualização"/>
+    <tableColumn id="19" name="O que a Prime Control faz bem hoje"/>
+    <tableColumn id="20" name="Soluções inovadoras e relevantes"/>
+    <tableColumn id="21" name="Expectativa sobre empresa inovadora"/>
+    <tableColumn id="22" name="Serviços conforme contratado"/>
+    <tableColumn id="23" name="Conhecimento do negócio"/>
+    <tableColumn id="24" name="Qualidade das entregas"/>
+    <tableColumn id="25" name="Informação sobre andamento e resultados"/>
+    <tableColumn id="26" name="Engajamento na solução de problemas"/>
+    <tableColumn id="27" name="Entregas dentro dos prazos"/>
+    <tableColumn id="28" name="Apresentações claras e relevantes"/>
+    <tableColumn id="29" name="Valor percebido"/>
+    <tableColumn id="30" name="Qualidade do atendimento"/>
+    <tableColumn id="31" name="Tempo de resposta da equipe"/>
+    <tableColumn id="32" name="Entregas, melhorias ou iniciativas para ampliar parceria"/>
+    <tableColumn id="33" name="Perguntas respondidas"/>
+    <tableColumn id="34" name="Campos abertos preenchidos"/>
+    <tableColumn id="35" name="Etapa abandonada"/>
+    <tableColumn id="36" name="Sinal de risco"/>
+    <tableColumn id="37" name="Status de follow-up"/>
+    <tableColumn id="38" name="Próxima ação"/>
+    <tableColumn id="39" name="Responsável follow-up"/>
+    <tableColumn id="40" name="Data follow-up"/>
+    <tableColumn id="41" name="Observações internas"/>
+    <tableColumn id="42" name="Link replay Clarity (opcional)"/>
+    <tableColumn id="43" name="Última atualização"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -751,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -852,7 +850,7 @@
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Leitura temática | 25% por bloco</t>
+          <t>Médias da avaliação | escala 1 a 5</t>
         </is>
       </c>
     </row>
@@ -880,12 +878,12 @@
       <c r="E12" s="9" t="n"/>
       <c r="F12" s="8" t="inlineStr">
         <is>
-          <t>Bloco</t>
+          <t>Dimensão</t>
         </is>
       </c>
       <c r="G12" s="8" t="inlineStr">
         <is>
-          <t>Peso</t>
+          <t>Escala</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr">
@@ -915,16 +913,16 @@
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
-          <t>Relacionamento e Satisfação</t>
+          <t>Inovação e relevância</t>
         </is>
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>1 a 5</t>
         </is>
       </c>
       <c r="H13" s="10">
-        <f>IFERROR(AVERAGE('Base automática'!Q:Q),"")</f>
+        <f>IFERROR(AVERAGE('Base automática'!T:T),"")</f>
         <v/>
       </c>
     </row>
@@ -949,16 +947,16 @@
       </c>
       <c r="F14" s="10" t="inlineStr">
         <is>
-          <t>Percepção de Valor</t>
+          <t>Execução contratada</t>
         </is>
       </c>
       <c r="G14" s="10" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>1 a 5</t>
         </is>
       </c>
       <c r="H14" s="10">
-        <f>IFERROR(SUM('Base automática'!T:X)/COUNT('Base automática'!T:X),"")</f>
+        <f>IFERROR(AVERAGE('Base automática'!V:V),"")</f>
         <v/>
       </c>
     </row>
@@ -970,7 +968,7 @@
       </c>
       <c r="B15" s="10" t="inlineStr">
         <is>
-          <t>Notas 1-6</t>
+          <t>Notas 0-6</t>
         </is>
       </c>
       <c r="C15" s="10">
@@ -983,16 +981,16 @@
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
-          <t>Qualidade Operacional</t>
+          <t>Conhecimento e parceria</t>
         </is>
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>1 a 5</t>
         </is>
       </c>
       <c r="H15" s="10">
-        <f>IFERROR(SUM('Base automática'!Y:AC)/COUNT('Base automática'!Y:AC),"")</f>
+        <f>IFERROR(SUM('Base automática'!W:W,'Base automática'!Z:Z)/COUNT('Base automática'!W:W,'Base automática'!Z:Z),"")</f>
         <v/>
       </c>
     </row>
@@ -1014,67 +1012,112 @@
       </c>
       <c r="F16" s="10" t="inlineStr">
         <is>
-          <t>Inovação, Transformação e Futuro</t>
+          <t>Entregas</t>
         </is>
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>1 a 5</t>
         </is>
       </c>
       <c r="H16" s="10">
-        <f>IFERROR(SUM('Base automática'!AD:AE)/COUNT('Base automática'!AD:AE),"")</f>
+        <f>IFERROR(SUM('Base automática'!X:X,'Base automática'!AA:AA)/COUNT('Base automática'!X:X,'Base automática'!AA:AA),"")</f>
         <v/>
       </c>
     </row>
-    <row r="17" ht="24" customHeight="1"/>
-    <row r="18" ht="24" customHeight="1"/>
+    <row r="17" ht="24" customHeight="1">
+      <c r="F17" s="10" t="inlineStr">
+        <is>
+          <t>Comunicação</t>
+        </is>
+      </c>
+      <c r="G17" s="10" t="inlineStr">
+        <is>
+          <t>1 a 5</t>
+        </is>
+      </c>
+      <c r="H17" s="10">
+        <f>IFERROR(SUM('Base automática'!Y:Y,'Base automática'!AB:AB)/COUNT('Base automática'!Y:Y,'Base automática'!AB:AB),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="F18" s="10" t="inlineStr">
+        <is>
+          <t>Valor percebido</t>
+        </is>
+      </c>
+      <c r="G18" s="10" t="inlineStr">
+        <is>
+          <t>1 a 5</t>
+        </is>
+      </c>
+      <c r="H18" s="10">
+        <f>IFERROR(AVERAGE('Base automática'!AC:AC),"")</f>
+        <v/>
+      </c>
+    </row>
     <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="7" t="inlineStr">
+      <c r="F19" s="10" t="inlineStr">
+        <is>
+          <t>Atendimento</t>
+        </is>
+      </c>
+      <c r="G19" s="10" t="inlineStr">
+        <is>
+          <t>1 a 5</t>
+        </is>
+      </c>
+      <c r="H19" s="10">
+        <f>IFERROR(AVERAGE('Base automática'!AD:AE),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20" ht="24" customHeight="1"/>
+    <row r="21" ht="24" customHeight="1"/>
+    <row r="22" ht="24" customHeight="1"/>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>Fluxo SharePoint/OneDrive</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="24" customHeight="1">
-      <c r="A20" s="12" t="inlineStr">
-        <is>
-          <t>1. Subir este arquivo no SharePoint/OneDrive da empresa.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="24" customHeight="1">
-      <c r="A21" s="12" t="inlineStr">
-        <is>
-          <t>2. Manter a aba Base automática como destino da integração.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="24" customHeight="1">
-      <c r="A22" s="12" t="inlineStr">
-        <is>
-          <t>3. A plataforma NPS grava respostas no Supabase e atualiza a planilha via Microsoft Graph API.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="12" t="inlineStr">
-        <is>
-          <t>4. O time pode criar análises manuais em novas abas sem alterar a Base automática.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="24" customHeight="1">
       <c r="A24" s="12" t="inlineStr">
         <is>
+          <t>1. Subir este arquivo no SharePoint/OneDrive da empresa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="12" t="inlineStr">
+        <is>
+          <t>2. Manter a aba Base automática como destino da integração.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="12" t="inlineStr">
+        <is>
+          <t>3. A plataforma NPS grava respostas no Supabase e atualiza a planilha via Microsoft Graph API.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="12" t="inlineStr">
+        <is>
+          <t>4. O time pode criar análises manuais em novas abas sem alterar a Base automática.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="12" t="inlineStr">
+        <is>
           <t>5. Heatmaps e replays continuam no Microsoft Clarity; a planilha recebe apenas link opcional quando houver análise manual.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1"/>
-    <row r="26" ht="24" customHeight="1"/>
-    <row r="27" ht="24" customHeight="1"/>
-    <row r="28" ht="24" customHeight="1"/>
     <row r="29" ht="24" customHeight="1"/>
     <row r="30" ht="24" customHeight="1"/>
     <row r="31" ht="24" customHeight="1"/>
@@ -1088,8 +1131,10 @@
     <mergeCell ref="G8:H8"/>
     <mergeCell ref="A7:B7"/>
     <mergeCell ref="G7:H7"/>
+    <mergeCell ref="A25:H25"/>
     <mergeCell ref="A11:D11"/>
-    <mergeCell ref="A21:H21"/>
+    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="A26:H26"/>
     <mergeCell ref="D7:E7"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A5:B5"/>
@@ -1098,13 +1143,11 @@
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A8:B8"/>
     <mergeCell ref="F11:H11"/>
-    <mergeCell ref="A22:H22"/>
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="G4:H4"/>
     <mergeCell ref="D8:E8"/>
-    <mergeCell ref="A20:H20"/>
     <mergeCell ref="D5:E5"/>
-    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A28:H28"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -1117,7 +1160,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS2"/>
+  <dimension ref="A1:AQ2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1250,7 +1293,7 @@
       </c>
       <c r="Q1" s="8" t="inlineStr">
         <is>
-          <t>Nota NPS (1 a 10)</t>
+          <t>Nota NPS (0 a 10)</t>
         </is>
       </c>
       <c r="R1" s="8" t="inlineStr">
@@ -1260,135 +1303,125 @@
       </c>
       <c r="S1" s="8" t="inlineStr">
         <is>
-          <t>Motivo da nota</t>
+          <t>O que a Prime Control faz bem hoje</t>
         </is>
       </c>
       <c r="T1" s="8" t="inlineStr">
         <is>
-          <t>Entendimento do negócio</t>
+          <t>Soluções inovadoras e relevantes</t>
         </is>
       </c>
       <c r="U1" s="8" t="inlineStr">
         <is>
-          <t>Relevância das soluções entregues</t>
+          <t>Expectativa sobre empresa inovadora</t>
         </is>
       </c>
       <c r="V1" s="8" t="inlineStr">
         <is>
+          <t>Serviços conforme contratado</t>
+        </is>
+      </c>
+      <c r="W1" s="8" t="inlineStr">
+        <is>
+          <t>Conhecimento do negócio</t>
+        </is>
+      </c>
+      <c r="X1" s="8" t="inlineStr">
+        <is>
+          <t>Qualidade das entregas</t>
+        </is>
+      </c>
+      <c r="Y1" s="8" t="inlineStr">
+        <is>
+          <t>Informação sobre andamento e resultados</t>
+        </is>
+      </c>
+      <c r="Z1" s="8" t="inlineStr">
+        <is>
+          <t>Engajamento na solução de problemas</t>
+        </is>
+      </c>
+      <c r="AA1" s="8" t="inlineStr">
+        <is>
+          <t>Entregas dentro dos prazos</t>
+        </is>
+      </c>
+      <c r="AB1" s="8" t="inlineStr">
+        <is>
+          <t>Apresentações claras e relevantes</t>
+        </is>
+      </c>
+      <c r="AC1" s="8" t="inlineStr">
+        <is>
           <t>Valor percebido</t>
         </is>
       </c>
-      <c r="W1" s="8" t="inlineStr">
-        <is>
-          <t>Comprometimento com resultados</t>
-        </is>
-      </c>
-      <c r="X1" s="8" t="inlineStr">
-        <is>
-          <t>Engajamento na solução de problemas</t>
-        </is>
-      </c>
-      <c r="Y1" s="8" t="inlineStr">
-        <is>
-          <t>Qualidade das entregas</t>
-        </is>
-      </c>
-      <c r="Z1" s="8" t="inlineStr">
-        <is>
-          <t>Cumprimento dos prazos</t>
-        </is>
-      </c>
-      <c r="AA1" s="8" t="inlineStr">
-        <is>
-          <t>Clareza e objetividade</t>
-        </is>
-      </c>
-      <c r="AB1" s="8" t="inlineStr">
+      <c r="AD1" s="8" t="inlineStr">
+        <is>
+          <t>Qualidade do atendimento</t>
+        </is>
+      </c>
+      <c r="AE1" s="8" t="inlineStr">
         <is>
           <t>Tempo de resposta da equipe</t>
         </is>
       </c>
-      <c r="AC1" s="8" t="inlineStr">
-        <is>
-          <t>Qualidade do atendimento</t>
-        </is>
-      </c>
-      <c r="AD1" s="8" t="inlineStr">
-        <is>
-          <t>Empresa inovadora e alinhada ao mercado</t>
-        </is>
-      </c>
-      <c r="AE1" s="8" t="inlineStr">
-        <is>
-          <t>Antecipar tendências e propor soluções</t>
-        </is>
-      </c>
       <c r="AF1" s="8" t="inlineStr">
         <is>
-          <t>Áreas para investir mais em inovação</t>
+          <t>Entregas, melhorias ou iniciativas para ampliar parceria</t>
         </is>
       </c>
       <c r="AG1" s="8" t="inlineStr">
         <is>
-          <t>Expectativa sobre parceria estratégica</t>
+          <t>Perguntas respondidas</t>
         </is>
       </c>
       <c r="AH1" s="8" t="inlineStr">
         <is>
-          <t>Iniciativas/melhorias para gerar mais valor</t>
+          <t>Campos abertos preenchidos</t>
         </is>
       </c>
       <c r="AI1" s="8" t="inlineStr">
         <is>
-          <t>Perguntas respondidas</t>
+          <t>Etapa abandonada</t>
         </is>
       </c>
       <c r="AJ1" s="8" t="inlineStr">
         <is>
-          <t>Campos abertos preenchidos</t>
+          <t>Sinal de risco</t>
         </is>
       </c>
       <c r="AK1" s="8" t="inlineStr">
         <is>
-          <t>Etapa abandonada</t>
+          <t>Status de follow-up</t>
         </is>
       </c>
       <c r="AL1" s="8" t="inlineStr">
         <is>
-          <t>Sinal de risco</t>
+          <t>Próxima ação</t>
         </is>
       </c>
       <c r="AM1" s="8" t="inlineStr">
         <is>
-          <t>Status de follow-up</t>
+          <t>Responsável follow-up</t>
         </is>
       </c>
       <c r="AN1" s="8" t="inlineStr">
         <is>
-          <t>Próxima ação</t>
+          <t>Data follow-up</t>
         </is>
       </c>
       <c r="AO1" s="8" t="inlineStr">
         <is>
-          <t>Responsável follow-up</t>
+          <t>Observações internas</t>
         </is>
       </c>
       <c r="AP1" s="8" t="inlineStr">
         <is>
-          <t>Data follow-up</t>
+          <t>Link replay Clarity (opcional)</t>
         </is>
       </c>
       <c r="AQ1" s="8" t="inlineStr">
-        <is>
-          <t>Observações internas</t>
-        </is>
-      </c>
-      <c r="AR1" s="8" t="inlineStr">
-        <is>
-          <t>Link replay Clarity (opcional)</t>
-        </is>
-      </c>
-      <c r="AS1" s="8" t="inlineStr">
         <is>
           <t>Última atualização</t>
         </is>
@@ -1438,11 +1471,9 @@
       <c r="AO2" s="10" t="inlineStr"/>
       <c r="AP2" s="10" t="inlineStr"/>
       <c r="AQ2" s="10" t="inlineStr"/>
-      <c r="AR2" s="10" t="inlineStr"/>
-      <c r="AS2" s="10" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AS1"/>
+  <autoFilter ref="A1:AQ1"/>
   <conditionalFormatting sqref="Q2:Q5000">
     <cfRule type="cellIs" priority="1" operator="lessThanOrEqual" dxfId="0">
       <formula>6</formula>
@@ -1913,7 +1944,7 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>Nota NPS (1 a 10)</t>
+          <t>Nota NPS (0 a 10)</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">

</xml_diff>